<commit_message>
Update Western Canada internships spreadsheet 2026-09-13
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Investment Management Intern, Canadian Equities</t>
+          <t>Test Developer Co-op</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,29 +535,29 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711073006</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Aug 26, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---Cloud--Data-and-AI---Summer-Intern---Calgary_752586WD</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711071006</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Mackenzie Investments</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Winter Intern, Investment Management, Multi-Asset</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,24 +599,24 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/May-2027---Cloud--Data-and-AI---Summer-Intern---Vancouver_752583WD</t>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/6008/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>Digital Hardware Engineer Intern</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---SAP---Summer-Intern---Calgary_752589WD</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
+          <t>Measurement Intern</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Fort-McMurray-Base-Plant-AB-CAN/Automation--Software-or-Computer-Engineering-Student---January-2027_R0017525</t>
+          <t>https://careers-canada-secure.icims.com/jobs/1954/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Data Science Student</t>
+          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://suncor.wd1.myworkdayjobs.com/Suncor_External/job/Calgary-AB-CAN/Data-Science-Student---January-2027_R0017534</t>
+          <t>https://careers-canada-secure.icims.com/jobs/1926/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Engineering Co-op, Electric Division</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Calgary, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,24 +727,24 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20508</t>
+          <t>https://careers-canada-secure.icims.com/jobs/1934/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Aug 11, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Intact</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Gears of War</t>
+          <t>AI Developer Intern Co-op</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -759,217 +759,1513 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556956276</t>
+          <t>https://intactfc.wd3.myworkdayjobs.com/en-US/intactfc/job/Vancouver-British-Columbia-CAN/AI-Developer---4-Month-Internship-Co-op--Winter-2027--_R155235</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>AI and Compiler Engineering Graduate Intern</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/AI-and-Compiler-Engineering-Graduate-Intern_JR0286850</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Sep 9, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Zaber Technologies</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Software Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Sep 8, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Zaber Technologies</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Embedded Software Co-op</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Sep 8, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Rivian and Volkswagen Group Technologies</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern, Vehicle Controls</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Sep 8, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ATCO</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Data Analytics Co-op, Customer Operations</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20626</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Sep 5, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Data Analytics Intern</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/super.com/68809622-6599-4379-bb88-925b2d8fcfd9/</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer in Data Intern</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/super.com/2c889dd2-0103-43e8-a405-e5b006d8b5ec/</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Platform</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/super.com/29751d58-eacc-4b5a-8e9d-e59cb7a595c7/</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Data Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/super.com/5251792e-093d-42c6-ae9e-08c656e90807/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Full-Stack</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/super.com/b2615f7e-c6d2-46d6-9699-5027da9b5757/</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Data Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/super.com/c54cf7df-73b3-49d4-acff-5dc04fba15a4/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>AltaML</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/altaml/1b27d80a-ac06-45cd-9335-37d9380226dd/</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>General Dynamics UK</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Domain System Engineering Co-op</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>AltaML</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Associate Software Developer</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB / Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/altaml/abed5ba5-8cbe-46b1-beae-25fe30bc4c91/</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>General Dynamics UK</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineering Co-op</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Hexagon AB</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Sensor Fusion Defence Intern</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3079/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Hexagon AB</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Defense Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Hexagon AB</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Geomatics Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3093/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Kinaxis</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Developer Intern Co-op, Machine Learning</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>https://careers-kinaxis.icims.com/jobs/35297/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>North American Construction Group</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Full Stack Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Acheson, AB</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>AltaML</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Associate Software Engineer</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Atlassian</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Varian</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Software Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-op---University-of-Manitoba_R-30141</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>General Dynamics UK</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Software Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Remarcable</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Full Stack Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Firmware Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90301?icims=1</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Firmware Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91313?icims=1</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91366?icims=1</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Product Management Intern/Co-op - Multiple Teams</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>AGS Libraries Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Mackenzie Investments</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Investment Management Intern, Canadian Equities</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Aug 26, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---Cloud--Data-and-AI---Summer-Intern---Calgary_752586WD</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/May-2027---Cloud--Data-and-AI---Summer-Intern---Vancouver_752583WD</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Summer Intern, SAP</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---SAP---Summer-Intern---Calgary_752589WD</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>Onware</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Full Stack Developer, Intern</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Edmonton, AB</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>https://ats.rippling.com/onware/jobs/1b9d59b6-1ab0-4c40-8429-39b5b62f019a</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Jul 21, 2026</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Motorola</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Data Analyst Co-op</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>Aug 24, 2026</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>CLEAResult</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Energy Efficiency Analyst Co-op</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Remote, Canada</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>Aug 24, 2026</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Data Science Student</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>ATCO</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Engineering Co-op, Electric Division</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Gears of War</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Aug 6, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Software Engineer Intern</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Vancouver, BC</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>Aug 2, 2026</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>British Columbia Investment</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Risk Analytics Solutions Co-op/Intern</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Victoria, BC</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>British Columbia Investment</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Risk Reporting &amp; Data Co-op/Internship</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Victoria, BC</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>British Columbia Investment</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>Data &amp; Analytics Engineer Co-op/Intern</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Victoria, BC / Vancouver, BC</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-09-20
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Test Developer Co-op</t>
+          <t>AI Co-op Student</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,29 +535,29 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711073006</t>
+          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Robotics Software Co-op</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711071006</t>
+          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Winter Intern, Investment Management, Multi-Asset</t>
+          <t>Investment Risk Analytics Solutions Co-op Intern</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,29 +599,29 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/6008/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Risk-Analytics-Solutions-Co-op-Internship--Winter-2027-_JR101608</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sep 10, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Digital Hardware Engineer Intern</t>
+          <t>AI and Automation Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/AI-and-Automation-Engineer-Co-op-Internship--Winter---Summer-2027-_JR101597-1</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Measurement Intern</t>
+          <t>Technology Solutions Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://careers-canada-secure.icims.com/jobs/1954/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Technology-Solutions-Engineer-Co-op-Internship--Winter-2027-_JR101601</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
+          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://careers-canada-secure.icims.com/jobs/1926/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Tech-Data---Analytics----Software-Engineer-Co-op-Internship--Winter-2027-or-Winter---Summer-2027-_JR101596</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Software Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,24 +727,24 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://careers-canada-secure.icims.com/jobs/1934/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Vancouver-BC/Software-Engineer-Co-op-Internship--Winter-2027-_JR101590</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Intact</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>AI Developer Intern Co-op</t>
+          <t>Software Developer Co-op, Full Stack</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -759,29 +759,29 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://intactfc.wd3.myworkdayjobs.com/en-US/intactfc/job/Vancouver-British-Columbia-CAN/AI-Developer---4-Month-Internship-Co-op--Winter-2027--_R155235</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>AI and Compiler Engineering Graduate Intern</t>
+          <t>Software Developer Co-op, C++</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -791,24 +791,24 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/AI-and-Compiler-Engineering-Graduate-Intern_JR0286850</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Machine Learning Applied Scientist Co-op</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -823,29 +823,29 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Co-op</t>
+          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -855,29 +855,29 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20646</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Rivian and Volkswagen Group Technologies</t>
+          <t>Nexthop.ai</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Vehicle Controls</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -887,29 +887,29 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
+          <t>https://nexthopai.bamboohr.com/careers/64/</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Co-op, Customer Operations</t>
+          <t>Software Development Engineer Co-op</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -919,29 +919,29 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20626</t>
+          <t>https://job-boards.greenhouse.io/athinkingape/jobs/8203048</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Sep 5, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/68809622-6599-4379-bb88-925b2d8fcfd9/</t>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>BDO Canada</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer in Data Intern</t>
+          <t>Data &amp; Analytics Co-op Intern</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -983,29 +983,29 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/2c889dd2-0103-43e8-a405-e5b006d8b5ec/</t>
+          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Platform</t>
+          <t>Test Developer Co-op</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1015,29 +1015,29 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/29751d58-eacc-4b5a-8e9d-e59cb7a595c7/</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711073006</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Data Engineer Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1047,29 +1047,29 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/5251792e-093d-42c6-ae9e-08c656e90807/</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711071006</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Mackenzie Investments</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Full-Stack</t>
+          <t>Winter Intern, Investment Management, Multi-Asset</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1079,29 +1079,29 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/b2615f7e-c6d2-46d6-9699-5027da9b5757/</t>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/6008/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Data Engineer Intern</t>
+          <t>Digital Hardware Engineer Intern</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1111,29 +1111,29 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/c54cf7df-73b3-49d4-acff-5dc04fba15a4/</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Measurement Intern</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1143,24 +1143,24 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/1b27d80a-ac06-45cd-9335-37d9380226dd/</t>
+          <t>https://careers-canada-secure.icims.com/jobs/1954/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Mobile Domain System Engineering Co-op</t>
+          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1175,29 +1175,29 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
+          <t>https://careers-canada-secure.icims.com/jobs/1926/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Associate Software Developer</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1207,29 +1207,29 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/abed5ba5-8cbe-46b1-beae-25fe30bc4c91/</t>
+          <t>https://careers-canada-secure.icims.com/jobs/1934/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Intact</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Co-op</t>
+          <t>AI Developer Intern Co-op</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1239,29 +1239,29 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
+          <t>https://intactfc.wd3.myworkdayjobs.com/en-US/intactfc/job/Vancouver-British-Columbia-CAN/AI-Developer---4-Month-Internship-Co-op--Winter-2027--_R155235</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Sensor Fusion Defence Intern</t>
+          <t>AI and Compiler Engineering Graduate Intern</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1271,29 +1271,29 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3079/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/AI-and-Compiler-Engineering-Graduate-Intern_JR0286850</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Defense Engineer Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1303,29 +1303,29 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Geomatics Engineer Intern</t>
+          <t>Embedded Software Co-op</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1335,29 +1335,29 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3093/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Kinaxis</t>
+          <t>Rivian and Volkswagen Group Technologies</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Developer Intern Co-op, Machine Learning</t>
+          <t>Software Engineering Intern, Vehicle Controls</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1367,29 +1367,29 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://careers-kinaxis.icims.com/jobs/35297/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>North American Construction Group</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>Data Analytics Co-op, Customer Operations</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Acheson, AB</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1399,12 +1399,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20626</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 5, 2026</t>
         </is>
       </c>
     </row>
@@ -1416,12 +1416,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Associate Software Engineer</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1431,29 +1431,29 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
+          <t>https://jobs.lever.co/altaml/1b27d80a-ac06-45cd-9335-37d9380226dd/</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Atlassian</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Mobile Domain System Engineering Co-op</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1463,29 +1463,29 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Associate Software Developer</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Calgary, AB / Edmonton, AB</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-op---University-of-Manitoba_R-30141</t>
+          <t>https://jobs.lever.co/altaml/abed5ba5-8cbe-46b1-beae-25fe30bc4c91/</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineering Co-op</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1527,29 +1527,29 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Remarcable</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>Sensor Fusion Defence Intern</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1559,29 +1559,29 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3079/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Defense Engineer Intern</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1591,29 +1591,29 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90301?icims=1</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Geomatics Engineer Intern</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1623,29 +1623,29 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91313?icims=1</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3093/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Kinaxis</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Developer Intern Co-op, Machine Learning</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1655,29 +1655,29 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91366?icims=1</t>
+          <t>https://careers-kinaxis.icims.com/jobs/35297/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>North American Construction Group</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Product Management Intern/Co-op - Multiple Teams</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Acheson, AB</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1687,29 +1687,29 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Engineer Intern/Co-op</t>
+          <t>Associate Software Engineer</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1719,29 +1719,29 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Atlassian</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1751,29 +1751,29 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>AGS Libraries Intern/Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1783,29 +1783,29 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-op---University-of-Manitoba_R-30141</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1815,29 +1815,29 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>Remarcable</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Investment Management Intern, Canadian Equities</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1847,29 +1847,29 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Aug 26, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1879,24 +1879,24 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---Cloud--Data-and-AI---Summer-Intern---Calgary_752586WD</t>
+          <t>https://careers.amd.com/jobs/90301?icims=1</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -1911,24 +1911,24 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Vancouver/May-2027---Cloud--Data-and-AI---Summer-Intern---Vancouver_752583WD</t>
+          <t>https://careers.amd.com/jobs/91313?icims=1</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -1943,229 +1943,253 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://pwc.wd3.myworkdayjobs.com/Global_Campus_Careers/job/Calgary/May-2027---SAP---Summer-Intern---Calgary_752589WD</t>
+          <t>https://careers.amd.com/jobs/91366?icims=1</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Product Management Intern/Co-op - Multiple Teams</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>AGS Libraries Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Mackenzie Investments</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Investment Management Intern, Canadian Equities</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Aug 26, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
           <t>Onware</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Full Stack Developer, Intern</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Edmonton, AB</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>https://ats.rippling.com/onware/jobs/1b9d59b6-1ab0-4c40-8429-39b5b62f019a</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>Jul 21, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>Motorola</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Data Analyst Co-op</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr"/>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Aug 24, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>CLEAResult</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>Energy Efficiency Analyst Co-op</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>Aug 24, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Suncor</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>Aug 17, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Suncor</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Data Science Student</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>Aug 17, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>ATCO</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>Engineering Co-op, Electric Division</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Edmonton, AB / Calgary, AB</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr"/>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>Aug 11, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer Intern, Gears of War</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>Aug 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -2176,24 +2200,24 @@
       <c r="E54" s="4" t="inlineStr"/>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Aug 2, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Risk Analytics Solutions Co-op/Intern</t>
+          <t>Software Engineer in Data Intern</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2204,24 +2228,24 @@
       <c r="E55" s="4" t="inlineStr"/>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+          <t>Software Engineer Intern, Platform</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2232,24 +2256,24 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC / Vancouver, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2260,12 +2284,432 @@
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="4" t="inlineStr">
         <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Full-Stack</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Data Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Toronto, ON / Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Motorola</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Data Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>CLEAResult</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Energy Efficiency Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Summer Intern, SAP</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Data Science Student</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>ATCO</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Engineering Co-op, Electric Division</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Gears of War</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Aug 6, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Aug 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Risk Analytics Solutions Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr"/>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr"/>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F57"/>
+  <autoFilter ref="A1:F72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-09-27
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>Cenovus Energy</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>AI Co-op Student</t>
+          <t>Information Technology Student (Summer 2027)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,29 +535,29 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
+          <t>https://cenovus.wd3.myworkdayjobs.com/careers/job/CA-AB-Calgary/Student--IT--Data-Science-and-Software--Calgary--May-2027-_R-411145</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>GoTo Group</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Robotics Software Co-op</t>
+          <t>Software Engineer Intern, C3PO</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
+          <t>https://goto.wd5.myworkdayjobs.com/GoToCareers/job/Remote-Canada/C3PO-Intern_R26-2245</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Investment Risk Analytics Solutions Co-op Intern</t>
+          <t>Data Analytics Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,29 +599,29 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Risk-Analytics-Solutions-Co-op-Internship--Winter-2027-_JR101608</t>
+          <t>https://jobs.ashbyhq.com/super.com/3ee6ff20-3502-410b-bf24-71db02488986/</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>AI and Automation Engineer Co-op Intern</t>
+          <t>System Simulation Co-op</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/AI-and-Automation-Engineer-Co-op-Internship--Winter---Summer-2027-_JR101597-1</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/System-Simulation-Engineering-CO-OP_JR0287122</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Technology Solutions Engineer Co-op/Intern</t>
+          <t>Firmware Development Undergraduate Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Technology-Solutions-Engineer-Co-op-Internship--Winter-2027-_JR101601</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Firmware-Development-Undergraduate-Engineering-Co-op_JR0286862</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Analog Devices</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
+          <t>Embedded Software Engineer Intern</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Toronto, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Tech-Data---Analytics----Software-Engineer-Co-op-Internship--Winter-2027-or-Winter---Summer-2027-_JR101596</t>
+          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/Canada-Toronto/Embedded-Software-Engineer_R266615</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern</t>
+          <t>Rendering Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,24 +727,24 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Vancouver-BC/Software-Engineer-Co-op-Internship--Winter-2027-_JR101590</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Rendering-Engineer-Intern/216222</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, Full Stack</t>
+          <t>AI Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -759,24 +759,24 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-Engineer/216236</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, C++</t>
+          <t>Software Engineer 1 Co-op, Data Foundations</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -791,24 +791,24 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
+          <t>https://careers.planview.com/jobs/5153?icims=1</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Applied Scientist Co-op</t>
+          <t>Software Engineer 1 Co-op, Flowplatform Team</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -823,29 +823,29 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
+          <t>https://careers.planview.com/jobs/5150?icims=1</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
+          <t>Software Engineer 1 Co-op, Portfolio Intelligence Team</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -855,29 +855,29 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20646</t>
+          <t>https://careers.planview.com/jobs/5151?icims=1</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Nexthop.ai</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineer 1 Co-op, Anvi</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -887,29 +887,29 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://nexthopai.bamboohr.com/careers/64/</t>
+          <t>https://careers.planview.com/jobs/5051?icims=1</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Co-op</t>
+          <t>Software Engineer 1 Co-op, Hub</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -919,29 +919,29 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/athinkingape/jobs/8203048</t>
+          <t>https://careers.planview.com/jobs/5152?icims=1</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineering Intern (Spring 2027)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
+          <t>https://job-boards.greenhouse.io/mercury/jobs/6199367004</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BDO Canada</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Co-op Intern</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -983,29 +983,29 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
+          <t>https://amazon.jobs/en/jobs/10553947/software-development-engineer-intern-summer-2027-can</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sep 14, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>TRC Companies</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Test Developer Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1015,29 +1015,29 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711073006</t>
+          <t>https://careers.trccompanies.com/jobs/26840?icims=1</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>AI Co-op Student</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1047,29 +1047,29 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711071006</t>
+          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Winter Intern, Investment Management, Multi-Asset</t>
+          <t>Robotics Software Co-op</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1079,29 +1079,29 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/6008/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sep 10, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Digital Hardware Engineer Intern</t>
+          <t>Investment Risk Analytics Solutions Co-op Intern</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1111,29 +1111,29 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Risk-Analytics-Solutions-Co-op-Internship--Winter-2027-_JR101608</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Measurement Intern</t>
+          <t>AI and Automation Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1143,29 +1143,29 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://careers-canada-secure.icims.com/jobs/1954/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/AI-and-Automation-Engineer-Co-op-Internship--Winter---Summer-2027-_JR101597-1</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
+          <t>Technology Solutions Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1175,29 +1175,29 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://careers-canada-secure.icims.com/jobs/1926/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Technology-Solutions-Engineer-Co-op-Internship--Winter-2027-_JR101601</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1207,29 +1207,29 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://careers-canada-secure.icims.com/jobs/1934/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Tech-Data---Analytics----Software-Engineer-Co-op-Internship--Winter-2027-or-Winter---Summer-2027-_JR101596</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Intact</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>AI Developer Intern Co-op</t>
+          <t>Software Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1239,29 +1239,29 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://intactfc.wd3.myworkdayjobs.com/en-US/intactfc/job/Vancouver-British-Columbia-CAN/AI-Developer---4-Month-Internship-Co-op--Winter-2027--_R155235</t>
+          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Vancouver-BC/Software-Engineer-Co-op-Internship--Winter-2027-_JR101590</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>AI and Compiler Engineering Graduate Intern</t>
+          <t>Software Developer Co-op, Full Stack</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1271,24 +1271,24 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/AI-and-Compiler-Engineering-Graduate-Intern_JR0286850</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Developer Co-op, C++</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1303,24 +1303,24 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Co-op</t>
+          <t>Machine Learning Applied Scientist Co-op</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1335,29 +1335,29 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Rivian and Volkswagen Group Technologies</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Vehicle Controls</t>
+          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1367,29 +1367,29 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20646</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Nexthop.ai</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Co-op, Customer Operations</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1399,29 +1399,29 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20626</t>
+          <t>https://nexthopai.bamboohr.com/careers/64/</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Sep 5, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Software Development Engineer Co-op</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1431,29 +1431,29 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/1b27d80a-ac06-45cd-9335-37d9380226dd/</t>
+          <t>https://job-boards.greenhouse.io/athinkingape/jobs/8203048</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Mobile Domain System Engineering Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1463,29 +1463,29 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>BDO Canada</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Associate Software Developer</t>
+          <t>Data &amp; Analytics Co-op Intern</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / Edmonton, AB</t>
+          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1495,29 +1495,29 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/abed5ba5-8cbe-46b1-beae-25fe30bc4c91/</t>
+          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Co-op</t>
+          <t>Test Developer Co-op</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1527,29 +1527,29 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711073006</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Sensor Fusion Defence Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1559,29 +1559,29 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3079/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711071006</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Mackenzie Investments</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Defense Engineer Intern</t>
+          <t>Winter Intern, Investment Management, Multi-Asset</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1591,12 +1591,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/6008/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 10, 2026</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Geomatics Engineer Intern</t>
+          <t>Digital Hardware Engineer Intern</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1623,29 +1623,29 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3093/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Kinaxis</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Developer Intern Co-op, Machine Learning</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1655,29 +1655,29 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://careers-kinaxis.icims.com/jobs/35297/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>North American Construction Group</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>Embedded Software Co-op</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Acheson, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1687,29 +1687,29 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>Rivian and Volkswagen Group Technologies</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Associate Software Engineer</t>
+          <t>Software Engineering Intern, Vehicle Controls</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1719,29 +1719,29 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
+          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Atlassian</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Mobile Domain System Engineering Co-op</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1751,29 +1751,29 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Associate Software Developer</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Calgary, AB / Edmonton, AB</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-op---University-of-Manitoba_R-30141</t>
+          <t>https://jobs.lever.co/altaml/abed5ba5-8cbe-46b1-beae-25fe30bc4c91/</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineering Co-op</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1815,29 +1815,29 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Remarcable</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>Sensor Fusion Defence Intern</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1847,29 +1847,29 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3079/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Defense Engineer Intern</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1879,29 +1879,29 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90301?icims=1</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Geomatics Engineer Intern</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1911,29 +1911,29 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91313?icims=1</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3093/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>North American Construction Group</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Acheson, AB</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1943,29 +1943,29 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91366?icims=1</t>
+          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Product Management Intern/Co-op - Multiple Teams</t>
+          <t>Associate Software Engineer</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1975,29 +1975,29 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Atlassian</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Engineer Intern/Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2007,29 +2007,29 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2039,24 +2039,24 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-op---University-of-Manitoba_R-30141</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>AGS Libraries Intern/Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2071,24 +2071,24 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Remarcable</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2103,29 +2103,29 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Investment Management Intern, Canadian Equities</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2135,29 +2135,29 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://careers.amd.com/jobs/90301?icims=1</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Aug 26, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Onware</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer, Intern</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2167,197 +2167,221 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/onware/jobs/1b9d59b6-1ab0-4c40-8429-39b5b62f019a</t>
+          <t>https://careers.amd.com/jobs/91313?icims=1</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Jul 21, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Data Analytics Intern</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Toronto, ON / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr"/>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>Sep 4, 2026</t>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Product Management Intern/Co-op - Multiple Teams</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer in Data Intern</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>Toronto, ON / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Sep 4, 2026</t>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer Intern, Platform</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>Toronto, ON / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr"/>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>Sep 4, 2026</t>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>Data Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>Toronto, ON / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>Sep 4, 2026</t>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>AGS Libraries Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer Intern, Full-Stack</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>Toronto, ON / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr"/>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Sep 4, 2026</t>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Data Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>Toronto, ON / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr"/>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Sep 4, 2026</t>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Mackenzie Investments</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Investment Management Intern, Canadian Equities</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Aug 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Data Analyst Co-op</t>
+          <t>Measurement Intern</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2368,24 +2392,24 @@
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>CLEAResult</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Energy Efficiency Analyst Co-op</t>
+          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2396,19 +2420,19 @@
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -2424,19 +2448,19 @@
       <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Intact</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>AI Developer Intern Co-op</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -2452,24 +2476,24 @@
       <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>AI and Compiler Engineering Graduate Intern</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2480,24 +2504,24 @@
       <c r="E64" s="4" t="inlineStr"/>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
+          <t>Data Analytics Co-op, Customer Operations</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2508,24 +2532,24 @@
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Data Science Student</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2536,24 +2560,24 @@
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Engineering Co-op, Electric Division</t>
+          <t>Software Engineer in Data Intern</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Calgary, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2564,24 +2588,24 @@
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Aug 11, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Gears of War</t>
+          <t>Software Engineer Intern, Platform</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2592,24 +2616,24 @@
       <c r="E68" s="4" t="inlineStr"/>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2620,24 +2644,24 @@
       <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Aug 2, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Risk Analytics Solutions Co-op/Intern</t>
+          <t>Software Engineer Intern, Full-Stack</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2648,24 +2672,24 @@
       <c r="E70" s="4" t="inlineStr"/>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2676,24 +2700,24 @@
       <c r="E71" s="4" t="inlineStr"/>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC / Vancouver, BC</t>
+          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2704,12 +2728,460 @@
       <c r="E72" s="4" t="inlineStr"/>
       <c r="F72" s="4" t="inlineStr">
         <is>
+          <t>Sep 4, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>Kinaxis</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Developer Intern Co-op, Machine Learning</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr"/>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>Motorola</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Data Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>CLEAResult</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Energy Efficiency Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr"/>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr"/>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Summer Intern, SAP</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Data Science Student</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>ATCO</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Engineering Co-op, Electric Division</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr"/>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Gears of War</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Aug 6, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr"/>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Aug 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Onware</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Full Stack Developer, Intern</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Jul 21, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Risk Analytics Solutions Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr"/>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr"/>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F72"/>
+  <autoFilter ref="A1:F88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-10-04
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cenovus Energy</t>
+          <t>Solink</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Information Technology Student (Summer 2027)</t>
+          <t>Software Engineer Co-op, Agents</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Ottawa, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,24 +535,24 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://cenovus.wd3.myworkdayjobs.com/careers/job/CA-AB-Calgary/Student--IT--Data-Science-and-Software--Calgary--May-2027-_R-411145</t>
+          <t>https://jobs.ashbyhq.com/solink/8493613d-ea47-4182-ac0b-f5f24d11f49e/</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sep 24, 2026</t>
+          <t>Oct 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GoTo Group</t>
+          <t>Kinaxis</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, C3PO</t>
+          <t>AI/ML Researcher Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://goto.wd5.myworkdayjobs.com/GoToCareers/job/Remote-Canada/C3PO-Intern_R26-2245</t>
+          <t>https://careers-kinaxis.icims.com/jobs/35465/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sep 24, 2026</t>
+          <t>Oct 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Intern (Winter 2027)</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,29 +599,29 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/super.com/3ee6ff20-3502-410b-bf24-71db02488986/</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/216227</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sep 23, 2026</t>
+          <t>Sep 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>System Simulation Co-op</t>
+          <t>Data Scientist Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/System-Simulation-Engineering-CO-OP_JR0287122</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4421775009</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sep 23, 2026</t>
+          <t>Sep 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Cenovus Energy</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Firmware Development Undergraduate Engineering Co-op (Winter 2027)</t>
+          <t>Information Technology Student (Summer 2027)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Firmware-Development-Undergraduate-Engineering-Co-op_JR0286862</t>
+          <t>https://cenovus.wd3.myworkdayjobs.com/careers/job/CA-AB-Calgary/Student--IT--Data-Science-and-Software--Calgary--May-2027-_R-411145</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sep 23, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Analog Devices</t>
+          <t>GoTo Group</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Engineer Intern</t>
+          <t>Software Engineer Intern, C3PO</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/Canada-Toronto/Embedded-Software-Engineer_R266615</t>
+          <t>https://goto.wd5.myworkdayjobs.com/GoToCareers/job/Remote-Canada/C3PO-Intern_R26-2245</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sep 23, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Rendering Engineer Intern (Summer 2027)</t>
+          <t>Firmware Development Undergraduate Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,29 +727,29 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Rendering-Engineer-Intern/216222</t>
+          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Firmware-Development-Undergraduate-Engineering-Co-op_JR0286862</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Analog Devices</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>AI Engineer Intern (Summer 2027)</t>
+          <t>Embedded Software Engineer Intern</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -759,24 +759,24 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-Engineer/216236</t>
+          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/Canada-Toronto/Embedded-Software-Engineer_R266615</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Data Foundations</t>
+          <t>Rendering Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://careers.planview.com/jobs/5153?icims=1</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Rendering-Engineer-Intern/216222</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -803,12 +803,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Flowplatform Team</t>
+          <t>AI Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://careers.planview.com/jobs/5150?icims=1</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-Engineer/216236</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -835,12 +835,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Portfolio Intelligence Team</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -855,29 +855,29 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://careers.planview.com/jobs/5151?icims=1</t>
+          <t>https://amazon.jobs/en/jobs/10553947/software-development-engineer-intern-summer-2027-can</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>TRC Companies</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Anvi</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -887,29 +887,29 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://careers.planview.com/jobs/5051?icims=1</t>
+          <t>https://careers.trccompanies.com/jobs/26840?icims=1</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Hub</t>
+          <t>AI Co-op Student</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -919,29 +919,29 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://careers.planview.com/jobs/5152?icims=1</t>
+          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Intern (Spring 2027)</t>
+          <t>Robotics Software Co-op</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -951,24 +951,24 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/mercury/jobs/6199367004</t>
+          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sep 21, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern</t>
+          <t>Software Developer Co-op, Full Stack</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -983,29 +983,29 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://amazon.jobs/en/jobs/10553947/software-development-engineer-intern-summer-2027-can</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sep 18, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TRC Companies</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Developer Co-op, C++</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1015,29 +1015,29 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://careers.trccompanies.com/jobs/26840?icims=1</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sep 18, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>AI Co-op Student</t>
+          <t>Machine Learning Applied Scientist Co-op</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1047,29 +1047,29 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Robotics Software Co-op</t>
+          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1079,29 +1079,29 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
+          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20646</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Nexthop.ai</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Investment Risk Analytics Solutions Co-op Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1111,29 +1111,29 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Risk-Analytics-Solutions-Co-op-Internship--Winter-2027-_JR101608</t>
+          <t>https://nexthopai.bamboohr.com/careers/64/</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>AI and Automation Engineer Co-op Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1143,29 +1143,29 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/AI-and-Automation-Engineer-Co-op-Internship--Winter---Summer-2027-_JR101597-1</t>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>BDO Canada</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Technology Solutions Engineer Co-op/Intern</t>
+          <t>Data &amp; Analytics Co-op Intern</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1175,29 +1175,29 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Technology-Solutions-Engineer-Co-op-Internship--Winter-2027-_JR101601</t>
+          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
+          <t>Digital Hardware Engineer Intern</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1207,29 +1207,29 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Victoria-BC/Investment-Tech-Data---Analytics----Software-Engineer-Co-op-Internship--Winter-2027-or-Winter---Summer-2027-_JR101596</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1239,24 +1239,24 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://bci.wd10.myworkdayjobs.com/BCI_Careers/job/Vancouver-BC/Software-Engineer-Co-op-Internship--Winter-2027-_JR101590</t>
+          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, Full Stack</t>
+          <t>Embedded Software Co-op</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1271,24 +1271,24 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
+          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Rivian and Volkswagen Group Technologies</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, C++</t>
+          <t>Software Engineering Intern, Vehicle Controls</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1303,29 +1303,29 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
+          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Applied Scientist Co-op</t>
+          <t>Mobile Domain System Engineering Co-op</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1335,29 +1335,29 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
+          <t>Software Engineering Co-op</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1367,29 +1367,29 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20646</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Nexthop.ai</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Defense Engineer Intern</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1399,29 +1399,29 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://nexthopai.bamboohr.com/careers/64/</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>North American Construction Group</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Co-op</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Acheson, AB</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1431,29 +1431,29 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/athinkingape/jobs/8203048</t>
+          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Associate Software Engineer</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1463,29 +1463,29 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
+          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BDO Canada</t>
+          <t>Atlassian</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Co-op Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
+          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1495,29 +1495,29 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
+          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Sep 14, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Test Developer Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1527,24 +1527,24 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711073006</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Remarcable</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1559,29 +1559,29 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/visiersolutionsinc/jobs/4711071006</t>
+          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Winter Intern, Investment Management, Multi-Asset</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1591,29 +1591,29 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/6008/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://careers.amd.com/jobs/90301?icims=1</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Sep 10, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Digital Hardware Engineer Intern</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1623,29 +1623,29 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://careers.amd.com/jobs/91313?icims=1</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Product Management Intern/Co-op - Multiple Teams</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1655,24 +1655,24 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
+          <t>https://careers.amd.com/jobs/90411?icims=1</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Co-op</t>
+          <t>Hardware Design Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1687,24 +1687,24 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
+          <t>https://careers.amd.com/jobs/90372?icims=1</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Rivian and Volkswagen Group Technologies</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Vehicle Controls</t>
+          <t>Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1719,24 +1719,24 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
+          <t>https://careers.amd.com/jobs/91367?icims=1</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Mobile Domain System Engineering Co-op</t>
+          <t>AGS Libraries Intern/Co-op</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1751,29 +1751,29 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
+          <t>https://careers.amd.com/jobs/90427?icims=1</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Associate Software Developer</t>
+          <t>Hardware Design Verification Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB / Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1783,29 +1783,29 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/abed5ba5-8cbe-46b1-beae-25fe30bc4c91/</t>
+          <t>https://careers.amd.com/jobs/91362?icims=1</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Mackenzie Investments</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Co-op</t>
+          <t>Investment Management Intern, Canadian Equities</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1815,556 +1815,488 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
+          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Aug 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Hexagon AB</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Sensor Fusion Defence Intern</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Calgary, AB</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3079/job?mobile=true&amp;needsRedirect=false</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>Sep 3, 2026</t>
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Data Analytics Intern (Winter 2027)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Hexagon AB</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Defense Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Calgary, AB</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Sep 3, 2026</t>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>System Simulation Co-op</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Hexagon AB</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Geomatics Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Calgary, AB</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3093/job?mobile=true&amp;needsRedirect=false</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Sep 3, 2026</t>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Planview</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer 1 Co-op, Data Foundations</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>North American Construction Group</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Full Stack Developer Co-op</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Acheson, AB</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Sep 3, 2026</t>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Planview</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer 1 Co-op, Flowplatform Team</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>AltaML</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Associate Software Engineer</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Edmonton, AB</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>Sep 3, 2026</t>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Planview</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer 1 Co-op, Portfolio Intelligence Team</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Atlassian</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineer Intern</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Sep 3, 2026</t>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Planview</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer 1 Co-op, Anvi</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Varian</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Planview</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer 1 Co-op, Hub</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Sep 22, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Mercury</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Spring 2027)</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Sep 21, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Investment Risk Analytics Solutions Co-op Intern</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Sep 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>AI and Automation Engineer Co-op Intern</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Sep 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Technology Solutions Engineer Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Sep 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Sep 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Co-op Intern</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Sep 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>A Thinking Ape</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Software Development Engineer Co-op</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Sep 15, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Visier Solutions</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Test Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Sep 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Visier Solutions</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>Software Developer Co-op</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Sep 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Mackenzie Investments</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Winter Intern, Investment Management, Multi-Asset</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Winnipeg, MB</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-op---University-of-Manitoba_R-30141</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>Sep 3, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>General Dynamics UK</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Software Developer Co-op</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Calgary, AB</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Sep 2, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Remarcable</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Full Stack Developer Co-op</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>Sep 2, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Firmware Engineer Intern/Co-op</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.amd.com/jobs/90301?icims=1</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Firmware Engineer Intern/Co-op</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.amd.com/jobs/91313?icims=1</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Product Management Intern/Co-op - Multiple Teams</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Calgary, AB</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.amd.com/jobs/90411?icims=1</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Hardware Design Engineer Intern/Co-op</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.amd.com/jobs/90372?icims=1</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineer Intern/Co-op</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.amd.com/jobs/91367?icims=1</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>AGS Libraries Intern/Co-op</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Calgary, AB</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.amd.com/jobs/90427?icims=1</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Hardware Design Verification Engineer Intern/Co-op</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>https://careers.amd.com/jobs/91362?icims=1</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Mackenzie Investments</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Investment Management Intern, Canadian Equities</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Winnipeg, MB</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>Aug 26, 2026</t>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Sep 10, 2026</t>
         </is>
       </c>
     </row>
@@ -2735,17 +2667,17 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Kinaxis</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern Co-op, Machine Learning</t>
+          <t>Associate Software Developer</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB / Edmonton, AB</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2763,12 +2695,12 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Sensor Fusion Defence Intern</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -2784,24 +2716,24 @@
       <c r="E74" s="4" t="inlineStr"/>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Data Analyst Co-op</t>
+          <t>Geomatics Engineer Intern</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2812,19 +2744,19 @@
       <c r="E75" s="4" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>CLEAResult</t>
+          <t>Kinaxis</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Energy Efficiency Analyst Co-op</t>
+          <t>Developer Intern Co-op, Machine Learning</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -2840,24 +2772,24 @@
       <c r="E76" s="4" t="inlineStr"/>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2868,24 +2800,24 @@
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2896,24 +2828,24 @@
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>Data Analyst Co-op</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2924,24 +2856,24 @@
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Aug 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>CLEAResult</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
+          <t>Energy Efficiency Analyst Co-op</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2952,24 +2884,24 @@
       <c r="E80" s="4" t="inlineStr"/>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Aug 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Data Science Student</t>
+          <t>Cloud, Data and AI Intern</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2980,24 +2912,24 @@
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Aug 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Engineering Co-op, Electric Division</t>
+          <t>Cloud, Data and AI Intern</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -3008,24 +2940,24 @@
       <c r="E82" s="4" t="inlineStr"/>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Aug 11, 2026</t>
+          <t>Aug 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>PwC</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Gears of War</t>
+          <t>Summer Intern, SAP</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -3036,24 +2968,24 @@
       <c r="E83" s="4" t="inlineStr"/>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Aug 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Suncor</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -3064,24 +2996,24 @@
       <c r="E84" s="4" t="inlineStr"/>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Aug 2, 2026</t>
+          <t>Aug 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Onware</t>
+          <t>Suncor</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Developer, Intern</t>
+          <t>Data Science Student</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3092,24 +3024,24 @@
       <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Jul 21, 2026</t>
+          <t>Aug 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Risk Analytics Solutions Co-op/Intern</t>
+          <t>Engineering Co-op, Electric Division</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Edmonton, AB / Calgary, AB</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -3120,24 +3052,24 @@
       <c r="E86" s="4" t="inlineStr"/>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Aug 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+          <t>Software Engineer Intern, Gears of War</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3148,24 +3080,24 @@
       <c r="E87" s="4" t="inlineStr"/>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Aug 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -3176,12 +3108,124 @@
       <c r="E88" s="4" t="inlineStr"/>
       <c r="F88" s="4" t="inlineStr">
         <is>
+          <t>Aug 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>Onware</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Full Stack Developer, Intern</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Jul 21, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Risk Analytics Solutions Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr"/>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr"/>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr"/>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F88"/>
+  <autoFilter ref="A1:F92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-10-11
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Solink</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op, Agents</t>
+          <t>Software Developer, Embedded Appliances Co-op</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Ottawa, ON / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -535,29 +535,29 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/solink/8493613d-ea47-4182-ac0b-f5f24d11f49e/</t>
+          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Vancouver-Canada/Software-Developer--Embedded-Appliances-Co-Op_R69581</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Oct 2, 2026</t>
+          <t>Oct 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kinaxis</t>
+          <t>The Semios Group</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Researcher Intern (Winter 2027)</t>
+          <t>Software Developer Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://careers-kinaxis.icims.com/jobs/35465/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://apply.workable.com/semios/j/4B5D1FB613/</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Oct 2, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>StackAdapt</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineer Backend Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,29 +599,29 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/216227</t>
+          <t>https://job-boards.greenhouse.io/stackadapt-confidential/jobs/4386552009</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sep 30, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Moment Energy</t>
+          <t>StackAdapt</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist Co-op (Winter 2027)</t>
+          <t>Machine Learning Engineer Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Surrey, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4421775009</t>
+          <t>https://job-boards.greenhouse.io/stackadapt-confidential/jobs/4397976009</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sep 26, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Cenovus Energy</t>
+          <t>Astera Labs</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Information Technology Student (Summer 2027)</t>
+          <t>Platform Applications Engineer Intern Co-op</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://cenovus.wd3.myworkdayjobs.com/careers/job/CA-AB-Calgary/Student--IT--Data-Science-and-Software--Calgary--May-2027-_R-411145</t>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4733856005</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sep 24, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GoTo Group</t>
+          <t>Astera Labs</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, C3PO</t>
+          <t>System Validation Engineer Intern</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://goto.wd5.myworkdayjobs.com/GoToCareers/job/Remote-Canada/C3PO-Intern_R26-2245</t>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4729021005</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sep 24, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Firmware Development Undergraduate Engineering Co-op (Winter 2027)</t>
+          <t>Firmware Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,29 +727,29 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://intel.wd1.myworkdayjobs.com/en-us/external/job/Virtual-Canada/Firmware-Development-Undergraduate-Engineering-Co-op_JR0286862</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4434575009</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sep 23, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Analog Devices</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Engineer Intern</t>
+          <t>Software Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -759,29 +759,29 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/Canada-Toronto/Embedded-Software-Engineer_R266615</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4434577009</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sep 23, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>AltaGas</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Rendering Engineer Intern (Summer 2027)</t>
+          <t>Data Analytics &amp; Process Automation Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -791,29 +791,29 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Rendering-Engineer-Intern/216222</t>
+          <t>https://wgl.wd5.myworkdayjobs.com/altagas/job/Calgary-AB/XMLNAME-2027-Data-Analytics---AltaGas---2027-Process-Automation-Co-op-Student_R7321-1</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Khan Academy</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>AI Engineer Intern (Summer 2027)</t>
+          <t>Software Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -823,29 +823,29 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-Engineer/216236</t>
+          <t>https://job-boards.greenhouse.io/khanacademy/jobs/8250259</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Semtech</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern</t>
+          <t>Software Developer Co-op, Web/Cloud Application</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -855,24 +855,24 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://amazon.jobs/en/jobs/10553947/software-development-engineer-intern-summer-2027-can</t>
+          <t>https://semtech.wd1.myworkdayjobs.com/SemtechCareers/job/CAN---Richmond-BC/Software-Developer---Web-Cloud-Application--Co-op_REQ3644</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Sep 18, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TRC Companies</t>
+          <t>AltaGas</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Digital Intern, NextGen AI &amp; Data (Winter 2027)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -887,29 +887,29 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://careers.trccompanies.com/jobs/26840?icims=1</t>
+          <t>https://wgl.wd5.myworkdayjobs.com/altagas/job/Calgary-AB/AltaGas---2027-Digital--NextGen-AI---Data--Intern_R7312</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sep 18, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>Kinaxis</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>AI Co-op Student</t>
+          <t>AI/ML Researcher Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -919,29 +919,29 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
+          <t>https://careers-kinaxis.icims.com/jobs/35465/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Robotics Software Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/216227</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, Full Stack</t>
+          <t>Data Scientist Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -983,29 +983,29 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4421775009</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Analog Devices</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, C++</t>
+          <t>Embedded Software Engineer Intern</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1015,24 +1015,24 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
+          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/Canada-Toronto/Embedded-Software-Engineer_R266615</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Applied Scientist Co-op</t>
+          <t>Rendering Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1047,29 +1047,29 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Rendering-Engineer-Intern/216222</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
+          <t>AI Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1079,29 +1079,29 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://eezy.fa.ca2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX/job/20646</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-Engineer/216236</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Nexthop.ai</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1111,19 +1111,19 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://nexthopai.bamboohr.com/careers/64/</t>
+          <t>https://amazon.jobs/en/jobs/10553947/software-development-engineer-intern-summer-2027-can</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>TRC Companies</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1143,29 +1143,29 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
+          <t>https://careers.trccompanies.com/jobs/26840?icims=1</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BDO Canada</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Co-op Intern</t>
+          <t>AI Co-op Student</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1175,29 +1175,29 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
+          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sep 14, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Digital Hardware Engineer Intern</t>
+          <t>Robotics Software Co-op</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1207,24 +1207,24 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Developer Co-op, Full Stack</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1239,24 +1239,24 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Co-op</t>
+          <t>Software Developer Co-op, C++</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1271,24 +1271,24 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Rivian and Volkswagen Group Technologies</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Vehicle Controls</t>
+          <t>Machine Learning Applied Scientist Co-op</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1303,29 +1303,29 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/rivianvw.tech/e00c49b7-44c1-4f0c-af3c-2c7a7402185b/</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Nexthop.ai</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Mobile Domain System Engineering Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1335,29 +1335,29 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
+          <t>https://nexthopai.bamboohr.com/careers/64/</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1367,29 +1367,29 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>BDO Canada</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Defense Engineer Intern</t>
+          <t>Data &amp; Analytics Co-op Intern</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1399,29 +1399,29 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3078/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>North American Construction Group</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>Digital Hardware Engineer Intern</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Acheson, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1431,29 +1431,29 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://careers-nacg.icims.com/jobs/17153/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Associate Software Engineer</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1463,29 +1463,29 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
+          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Atlassian</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Embedded Software Co-op</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1495,12 +1495,12 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
+          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Mobile Domain System Engineering Co-op</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1527,29 +1527,29 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Remarcable</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>Software Engineering Co-op</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1559,29 +1559,29 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Associate Software Engineer</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1591,29 +1591,29 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90301?icims=1</t>
+          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Atlassian</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1623,24 +1623,24 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91313?icims=1</t>
+          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>General Dynamics UK</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Product Management Intern/Co-op - Multiple Teams</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1655,24 +1655,24 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Remarcable</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Engineer Intern/Co-op</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+          <t>https://careers.amd.com/jobs/90301?icims=1</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>AGS Libraries Intern/Co-op</t>
+          <t>Firmware Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+          <t>https://careers.amd.com/jobs/91313?icims=1</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1768,12 +1768,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+          <t>Product Management Intern/Co-op - Multiple Teams</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+          <t>https://careers.amd.com/jobs/90411?icims=1</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1795,161 +1795,177 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>AGS Libraries Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>Mackenzie Investments</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Investment Management Intern, Canadian Equities</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Winnipeg, MB</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Aug 26, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Data Analytics Intern (Winter 2027)</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>System Simulation Co-op</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Planview</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer 1 Co-op, Data Foundations</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>Planview</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer 1 Co-op, Flowplatform Team</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr"/>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>GoTo Group</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Portfolio Intelligence Team</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1960,24 +1976,24 @@
       <c r="E47" s="4" t="inlineStr"/>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>Solink</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Anvi</t>
+          <t>Software Engineer Co-op, Agents</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Ottawa, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1988,24 +2004,24 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Oct 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Planview</t>
+          <t>Cenovus Energy</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer 1 Co-op, Hub</t>
+          <t>Information Technology Student (Summer 2027)</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -2016,19 +2032,19 @@
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>GoTo Group</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern (Spring 2027)</t>
+          <t>Software Engineer Intern, C3PO</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -2044,24 +2060,24 @@
       <c r="E50" s="4" t="inlineStr"/>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Sep 21, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Investment Risk Analytics Solutions Co-op Intern</t>
+          <t>Data Analytics Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2072,24 +2088,24 @@
       <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>AI and Automation Engineer Co-op Intern</t>
+          <t>System Simulation Co-op</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2100,24 +2116,24 @@
       <c r="E52" s="4" t="inlineStr"/>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Technology Solutions Engineer Co-op/Intern</t>
+          <t>Firmware Development Undergraduate Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2128,24 +2144,24 @@
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
+          <t>Software Engineer 1 Co-op, Data Foundations</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -2156,24 +2172,24 @@
       <c r="E54" s="4" t="inlineStr"/>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern</t>
+          <t>Software Engineer 1 Co-op, Flowplatform Team</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2184,24 +2200,24 @@
       <c r="E55" s="4" t="inlineStr"/>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Co-op</t>
+          <t>Software Engineer 1 Co-op, Portfolio Intelligence Team</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2212,19 +2228,19 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Test Developer Co-op</t>
+          <t>Software Engineer 1 Co-op, Anvi</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -2240,19 +2256,19 @@
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Software Engineer 1 Co-op, Hub</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -2268,24 +2284,24 @@
       <c r="E58" s="4" t="inlineStr"/>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Winter Intern, Investment Management, Multi-Asset</t>
+          <t>Software Engineering Intern (Spring 2027)</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2296,24 +2312,24 @@
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Sep 10, 2026</t>
+          <t>Sep 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Measurement Intern</t>
+          <t>Investment Risk Analytics Solutions Co-op Intern</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2324,24 +2340,24 @@
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
+          <t>AI and Automation Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2352,24 +2368,24 @@
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Technology Solutions Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2380,24 +2396,24 @@
       <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Intact</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>AI Developer Intern Co-op</t>
+          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2408,24 +2424,24 @@
       <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>AI and Compiler Engineering Graduate Intern</t>
+          <t>Software Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2436,7 +2452,7 @@
       <c r="E64" s="4" t="inlineStr"/>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2464,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics Co-op, Customer Operations</t>
+          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -2464,24 +2480,24 @@
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Sep 5, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics Intern</t>
+          <t>Software Development Engineer Co-op</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2492,24 +2508,24 @@
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer in Data Intern</t>
+          <t>Test Developer Co-op</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2520,24 +2536,24 @@
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Platform</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2548,24 +2564,24 @@
       <c r="E68" s="4" t="inlineStr"/>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Mackenzie Investments</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Data Engineer Intern</t>
+          <t>Winter Intern, Investment Management, Multi-Asset</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2576,24 +2592,24 @@
       <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Full-Stack</t>
+          <t>Measurement Intern</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2604,24 +2620,24 @@
       <c r="E70" s="4" t="inlineStr"/>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Data Engineer Intern</t>
+          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2632,24 +2648,24 @@
       <c r="E71" s="4" t="inlineStr"/>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2660,24 +2676,24 @@
       <c r="E72" s="4" t="inlineStr"/>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>Intact</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Associate Software Developer</t>
+          <t>AI Developer Intern Co-op</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2688,24 +2704,24 @@
       <c r="E73" s="4" t="inlineStr"/>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Sensor Fusion Defence Intern</t>
+          <t>AI and Compiler Engineering Graduate Intern</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2716,24 +2732,24 @@
       <c r="E74" s="4" t="inlineStr"/>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Rivian and Volkswagen Group Technologies</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Geomatics Engineer Intern</t>
+          <t>Software Engineering Intern, Vehicle Controls</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2744,24 +2760,24 @@
       <c r="E75" s="4" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Kinaxis</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern Co-op, Machine Learning</t>
+          <t>Data Analytics Co-op, Customer Operations</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2772,24 +2788,24 @@
       <c r="E76" s="4" t="inlineStr"/>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2800,24 +2816,24 @@
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Software Engineer in Data Intern</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2828,24 +2844,24 @@
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Data Analyst Co-op</t>
+          <t>Software Engineer Intern, Platform</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2856,24 +2872,24 @@
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>CLEAResult</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Energy Efficiency Analyst Co-op</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2884,24 +2900,24 @@
       <c r="E80" s="4" t="inlineStr"/>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Software Engineer Intern, Full-Stack</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2912,24 +2928,24 @@
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2940,24 +2956,24 @@
       <c r="E82" s="4" t="inlineStr"/>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2968,24 +2984,24 @@
       <c r="E83" s="4" t="inlineStr"/>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
+          <t>Associate Software Developer</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Calgary, AB / Edmonton, AB</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -2996,24 +3012,24 @@
       <c r="E84" s="4" t="inlineStr"/>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Data Science Student</t>
+          <t>Sensor Fusion Defence Intern</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3024,24 +3040,24 @@
       <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Engineering Co-op, Electric Division</t>
+          <t>Defense Engineer Intern</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Calgary, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -3052,24 +3068,24 @@
       <c r="E86" s="4" t="inlineStr"/>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Aug 11, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Gears of War</t>
+          <t>Geomatics Engineer Intern</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3080,24 +3096,24 @@
       <c r="E87" s="4" t="inlineStr"/>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Kinaxis</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Developer Intern Co-op, Machine Learning</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -3108,24 +3124,24 @@
       <c r="E88" s="4" t="inlineStr"/>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Aug 2, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>Onware</t>
+          <t>North American Construction Group</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Developer, Intern</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Acheson, AB</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3136,24 +3152,24 @@
       <c r="E89" s="4" t="inlineStr"/>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Jul 21, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Risk Analytics Solutions Co-op/Intern</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -3164,24 +3180,24 @@
       <c r="E90" s="4" t="inlineStr"/>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+          <t>Software Engineer Intern/Co-op</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3192,24 +3208,24 @@
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+          <t>Data Analyst Co-op</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC / Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -3220,12 +3236,376 @@
       <c r="E92" s="4" t="inlineStr"/>
       <c r="F92" s="4" t="inlineStr">
         <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>CLEAResult</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Energy Efficiency Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr"/>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr"/>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr"/>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Summer Intern, SAP</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr"/>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr"/>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>Data Science Student</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr"/>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>ATCO</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Engineering Co-op, Electric Division</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr"/>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Gears of War</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr"/>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>Aug 6, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr"/>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>Aug 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>Onware</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>Full Stack Developer, Intern</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr"/>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>Jul 21, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>Risk Analytics Solutions Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr"/>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr"/>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr"/>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F92"/>
+  <autoFilter ref="A1:F105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Western Canada internships spreadsheet 2026-10-18
</commit_message>
<xml_diff>
--- a/western_canada_internships.xlsx
+++ b/western_canada_internships.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Western Canada Internships" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Western Canada Internships'!$A$1:$F$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -515,12 +515,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Software Developer, Embedded Appliances Co-op</t>
+          <t>Analytics Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -535,24 +535,24 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers/job/Vancouver-Canada/Software-Developer--Embedded-Appliances-Co-Op_R69581</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Analytics-Intern/216232</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Oct 7, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>The Semios Group</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op (Winter 2027)</t>
+          <t>AI/ML Software Engineer Co-op Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -567,29 +567,29 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/semios/j/4B5D1FB613/</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-ML-Software-Engineer-Intern-Summer-2027-8-Months-Masters-QVS/216234</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>StackAdapt</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Backend Intern (Winter 2027)</t>
+          <t>Test Engineering Co-op</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -599,29 +599,29 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/stackadapt-confidential/jobs/4386552009</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4455115009</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>StackAdapt</t>
+          <t>BC Pensions</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer Intern (Winter 2027)</t>
+          <t>Application Developer Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -631,29 +631,29 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/stackadapt-confidential/jobs/4397976009</t>
+          <t>https://fa-exby-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1013/job/227</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Astera Labs</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Platform Applications Engineer Intern Co-op</t>
+          <t>Data Science Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Vancouver, BC / Richmond, BC</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4733856005</t>
+          <t>https://boeing.wd1.myworkdayjobs.com/external_subsidiary/job/CAN---Richmond-Canada/Data-Science-Intern_JR2026526159</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Astera Labs</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>System Validation Engineer Intern</t>
+          <t>Data Science Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -695,29 +695,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4729021005</t>
+          <t>https://job-boards.greenhouse.io/later/jobs/8889650002</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Moment Energy</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineering Co-op (Winter 2027)</t>
+          <t>Software Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Surrey, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -727,29 +727,29 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4434575009</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/216287</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Moment Energy</t>
+          <t>Astera Labs</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Co-op (Winter 2027)</t>
+          <t>Firmware Engineer Co-op Intern (Spring 2027)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Surrey, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -759,29 +759,29 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4434577009</t>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4739544005</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AltaGas</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics &amp; Process Automation Co-op (Winter 2027)</t>
+          <t>Technical Artist Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -791,24 +791,24 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://wgl.wd5.myworkdayjobs.com/altagas/job/Calgary-AB/XMLNAME-2027-Data-Analytics---AltaGas---2027-Process-Automation-Co-op-Student_R7321-1</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Technical-Artist-Co-op/216406</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Oct 6, 2026</t>
+          <t>Oct 13, 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Khan Academy</t>
+          <t>1Password</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern (Summer 2027)</t>
+          <t>Data Intern, Product Analytics (Winter 2027)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -823,29 +823,29 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/khanacademy/jobs/8250259</t>
+          <t>https://jobs.ashbyhq.com/1password/412c1aac-13ce-4cc9-9c81-90a9a7a2ee48/</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Oct 5, 2026</t>
+          <t>Oct 12, 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, Web/Cloud Application</t>
+          <t>Software Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Richmond, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -855,29 +855,29 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://semtech.wd1.myworkdayjobs.com/SemtechCareers/job/CAN---Richmond-BC/Software-Developer---Web-Cloud-Application--Co-op_REQ3644</t>
+          <t>https://www.databricks.com/company/careers/university-recruiting---engineering/software-engineering-intern-2027-6865687002</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Oct 5, 2026</t>
+          <t>Oct 12, 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AltaGas</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Digital Intern, NextGen AI &amp; Data (Winter 2027)</t>
+          <t>Software Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -887,29 +887,29 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://wgl.wd5.myworkdayjobs.com/altagas/job/Calgary-AB/AltaGas---2027-Digital--NextGen-AI---Data--Intern_R7312</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern-Summer-2027-8-Months-Sports-Technology/216225</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Oct 5, 2026</t>
+          <t>Oct 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Kinaxis</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>AI/ML Researcher Intern (Winter 2027)</t>
+          <t>C++ Generalist Software Engineer Co-op (Summer 2027)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -919,12 +919,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://careers-kinaxis.icims.com/jobs/35465/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Co-op/216231</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Oct 2, 2026</t>
+          <t>Oct 9, 2026</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Gameplay Software Engineer Co-op (Summer 2027)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -951,29 +951,29 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/216227</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Co-op/216230</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sep 30, 2026</t>
+          <t>Oct 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Moment Energy</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Data Scientist Co-op (Winter 2027)</t>
+          <t>C++ Software Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Surrey, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -983,29 +983,29 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4421775009</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern-Summer-2027-8-months-UFC/216226</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sep 26, 2026</t>
+          <t>Oct 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Analog Devices</t>
+          <t>Workday</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Engineer Intern</t>
+          <t>Software Development Engineer Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Toronto, ON / Vancouver, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1015,24 +1015,24 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/Canada-Toronto/Embedded-Software-Engineer_R266615</t>
+          <t>https://workday.wd5.myworkdayjobs.com/Workday_Early_Career/job/Canada-BC-Vancouver/Software-Development-Engineer-Intern_JR-0110807</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sep 23, 2026</t>
+          <t>Oct 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Workday</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Rendering Engineer Intern (Summer 2027)</t>
+          <t>Product Manager Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1047,29 +1047,29 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/Rendering-Engineer-Intern/216222</t>
+          <t>https://workday.wd5.myworkdayjobs.com/Workday_Early_Career/job/Canada-BC-Vancouver/Product-Manager-Intern_JR-0110808</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Oct 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>AI Engineer Intern (Summer 2027)</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1079,24 +1079,24 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-Engineer/216236</t>
+          <t>https://onehealthineers.wd3.myworkdayjobs.com/SHSJB/job/YWG-BW/Software-Developer-Co-op---Red-River-College_R-30142</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sep 22, 2026</t>
+          <t>Oct 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>The Semios Group</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Software Development Engineer Intern</t>
+          <t>Software Developer Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1111,29 +1111,29 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://amazon.jobs/en/jobs/10553947/software-development-engineer-intern-summer-2027-can</t>
+          <t>https://apply.workable.com/semios/j/4B5D1FB613/</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Sep 18, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TRC Companies</t>
+          <t>Astera Labs</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Platform Applications Engineer Intern Co-op</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1143,29 +1143,29 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://careers.trccompanies.com/jobs/26840?icims=1</t>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4733856005</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Sep 18, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>Astera Labs</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>AI Co-op Student</t>
+          <t>System Validation Engineer Intern</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1175,29 +1175,29 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4729021005</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>4AG Robotics</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Robotics Software Co-op</t>
+          <t>Firmware Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Salmon Arm, BC</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1207,29 +1207,29 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4434575009</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, Full Stack</t>
+          <t>Software Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1239,29 +1239,29 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4434577009</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>AltaGas</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op, C++</t>
+          <t>Data Analytics &amp; Process Automation Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1271,29 +1271,29 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
+          <t>https://wgl.wd5.myworkdayjobs.com/altagas/job/Calgary-AB/XMLNAME-2027-Data-Analytics---AltaGas---2027-Process-Automation-Co-op-Student_R7321-1</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Apera AI</t>
+          <t>Semtech</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning Applied Scientist Co-op</t>
+          <t>Software Developer Co-op, Web/Cloud Application</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Richmond, BC</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1303,29 +1303,29 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
+          <t>https://semtech.wd1.myworkdayjobs.com/SemtechCareers/job/CAN---Richmond-BC/Software-Developer---Web-Cloud-Application--Co-op_REQ3644</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Sep 16, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Nexthop.ai</t>
+          <t>AltaGas</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Digital Intern, NextGen AI &amp; Data (Winter 2027)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1335,29 +1335,29 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://nexthopai.bamboohr.com/careers/64/</t>
+          <t>https://wgl.wd5.myworkdayjobs.com/altagas/job/Calgary-AB/AltaGas---2027-Digital--NextGen-AI---Data--Intern_R7312</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Kinaxis</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>AI/ML Researcher Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1367,29 +1367,29 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
+          <t>https://careers-kinaxis.icims.com/jobs/35465/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Oct 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BDO Canada</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Co-op Intern</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1399,29 +1399,29 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Software-Engineer-Intern/216227</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Sep 14, 2026</t>
+          <t>Sep 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Moment Energy</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Digital Hardware Engineer Intern</t>
+          <t>Data Scientist Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Surrey, BC</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1431,29 +1431,29 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://job-boards.greenhouse.io/momentenergy/jobs/4421775009</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 26, 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>Analog Devices</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Embedded Software Engineer Intern</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Vancouver, BC</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1463,24 +1463,24 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
+          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/Canada-Toronto/Embedded-Software-Engineer_R266615</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Zaber Technologies</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Embedded Software Co-op</t>
+          <t>Rendering Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1495,29 +1495,29 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/Rendering-Engineer-Intern/216222</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Mobile Domain System Engineering Co-op</t>
+          <t>AI Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1527,29 +1527,29 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
+          <t>https://jobs.ea.com/en_US/careers/JobDetail/AI-Engineer/216236</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Software Engineering Co-op</t>
+          <t>Software Development Engineer Intern</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1559,29 +1559,29 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
+          <t>https://amazon.jobs/en/jobs/10553947/software-development-engineer-intern-summer-2027-can</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>TRC Companies</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Associate Software Engineer</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1591,29 +1591,29 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
+          <t>https://careers.trccompanies.com/jobs/26840?icims=1</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 18, 2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Atlassian</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>AI Co-op Student</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1623,29 +1623,29 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
+          <t>https://ats.rippling.com/4ag/jobs/921801f5-ae83-4a49-a234-221a87d94fe7</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics UK</t>
+          <t>4AG Robotics</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>Robotics Software Co-op</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Salmon Arm, BC</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1655,24 +1655,24 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
+          <t>https://ats.rippling.com/4ag/jobs/71d97d10-87f2-4f53-88b7-97f27f392d24</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Remarcable</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>Software Developer Co-op, Full Stack</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1687,24 +1687,24 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/remarcable-inc/a4f3aaaa-9469-42e8-a610-450d25eb5da7/</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5240259007</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Sep 2, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Software Developer Co-op, C++</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1719,24 +1719,24 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90301?icims=1</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239394007</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Apera AI</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Firmware Engineer Intern/Co-op</t>
+          <t>Machine Learning Applied Scientist Co-op</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1751,29 +1751,29 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91313?icims=1</t>
+          <t>https://job-boards.greenhouse.io/aperaaiinc/jobs/5239440007</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 16, 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Nexthop.ai</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Product Management Intern/Co-op - Multiple Teams</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Burnaby, BC</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1783,24 +1783,24 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+          <t>https://nexthopai.bamboohr.com/careers/64/</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Engineer Intern/Co-op</t>
+          <t>Software Engineer Intern</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1815,29 +1815,29 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393556991773?hl=en</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>BDO Canada</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Data &amp; Analytics Co-op Intern</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Montreal, QC / Toronto, ON / Calgary, AB / Halifax, NS / Vancouver, BC / Oakville, ON / Ottawa, ON</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1847,24 +1847,24 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+          <t>https://bdo.wd3.myworkdayjobs.com/BDO/job/Toronto---Bay-St/Co-op-or-Intern--Data---Analytics--January-2027-_JR7061</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 14, 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>AGS Libraries Intern/Co-op</t>
+          <t>Digital Hardware Engineer Intern</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -1879,24 +1879,24 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+          <t>https://careers-hexagonpositioning.icims.com/jobs/3090/job?mobile=true&amp;needsRedirect=false</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -1911,29 +1911,29 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+          <t>https://apply.workable.com/zaber/j/EAB5877DC3/</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>Zaber Technologies</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Investment Management Intern, Canadian Equities</t>
+          <t>Embedded Software Co-op</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1943,365 +1943,413 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://careersen-mackenzieinvestments.icims.com/jobs/5993/job?mobile=true&amp;needsRedirect=false</t>
+          <t>https://apply.workable.com/zaber/j/1F627CC2BB/</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Aug 26, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>GoTo Group</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Software Developer Intern</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Oct 5, 2026</t>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>General Dynamics UK</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Domain System Engineering Co-op</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147552960</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>Solink</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer Co-op, Agents</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Ottawa, ON / Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr"/>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Oct 2, 2026</t>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>General Dynamics UK</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineering Co-op</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000147563929</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>Cenovus Energy</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology Student (Summer 2027)</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>AltaML</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Associate Software Engineer</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/altaml/bd8167f5-e84c-48b1-9cad-2831bf71dea1/</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Atlassian</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Burnaby, BC / Vancouver, BC / Richmond, BC</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>https://campus-globalcareers-atlassian.icims.com/jobs/26275/software-engineer-intern%2c-2027-canada/job</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>General Dynamics UK</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Software Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Calgary, AB</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>Sep 24, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>GoTo Group</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer Intern, C3PO</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>Sep 24, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Super</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Data Analytics Intern (Winter 2027)</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/GDMSI/744000146985399</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>System Simulation Co-op</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr"/>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Firmware Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90301?icims=1</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Firmware Development Undergraduate Engineering Co-op (Winter 2027)</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>Remote, Canada</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>Sep 23, 2026</t>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Firmware Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91313?icims=1</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Planview</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer 1 Co-op, Data Foundations</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr"/>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Product Management Intern/Co-op - Multiple Teams</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90411?icims=1</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>Planview</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer 1 Co-op, Flowplatform Team</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90372?icims=1</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>Planview</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer 1 Co-op, Portfolio Intelligence Team</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr"/>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91367?icims=1</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Planview</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer 1 Co-op, Anvi</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>AGS Libraries Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/90427?icims=1</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>Planview</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>Software Engineer 1 Co-op, Hub</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver, BC</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr"/>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Sep 22, 2026</t>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Hardware Design Verification Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.amd.com/jobs/91362?icims=1</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Motorola</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern (Spring 2027)</t>
+          <t>Software Developer, Embedded Appliances Co-op</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2312,24 +2360,24 @@
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Sep 21, 2026</t>
+          <t>Oct 7, 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>StackAdapt</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Investment Risk Analytics Solutions Co-op Intern</t>
+          <t>Software Engineer Backend Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2340,24 +2388,24 @@
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>StackAdapt</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>AI and Automation Engineer Co-op Intern</t>
+          <t>Machine Learning Engineer Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2368,24 +2416,24 @@
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 6, 2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Khan Academy</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Technology Solutions Engineer Co-op/Intern</t>
+          <t>Software Engineer Intern (Summer 2027)</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2396,24 +2444,24 @@
       <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>GoTo Group</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2424,24 +2472,24 @@
       <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Solink</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Co-op Intern</t>
+          <t>Software Engineer Co-op, Agents</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Ottawa, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2452,24 +2500,24 @@
       <c r="E64" s="4" t="inlineStr"/>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Sep 17, 2026</t>
+          <t>Oct 2, 2026</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>Cenovus Energy</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
+          <t>Information Technology Student (Summer 2027)</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2480,19 +2528,19 @@
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>A Thinking Ape</t>
+          <t>GoTo Group</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Software Development Engineer Co-op</t>
+          <t>Software Engineer Intern, C3PO</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -2508,24 +2556,24 @@
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Sep 15, 2026</t>
+          <t>Sep 24, 2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Test Developer Co-op</t>
+          <t>Data Analytics Intern (Winter 2027)</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2536,24 +2584,24 @@
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Visier Solutions</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>System Simulation Co-op</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2564,24 +2612,24 @@
       <c r="E68" s="4" t="inlineStr"/>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Sep 11, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Mackenzie Investments</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Winter Intern, Investment Management, Multi-Asset</t>
+          <t>Firmware Development Undergraduate Engineering Co-op (Winter 2027)</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2592,24 +2640,24 @@
       <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Sep 10, 2026</t>
+          <t>Sep 23, 2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Measurement Intern</t>
+          <t>Software Engineer 1 Co-op, Data Foundations</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2620,24 +2668,24 @@
       <c r="E70" s="4" t="inlineStr"/>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
+          <t>Software Engineer 1 Co-op, Flowplatform Team</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2648,24 +2696,24 @@
       <c r="E71" s="4" t="inlineStr"/>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Intern</t>
+          <t>Software Engineer 1 Co-op, Portfolio Intelligence Team</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2676,19 +2724,19 @@
       <c r="E72" s="4" t="inlineStr"/>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Intact</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>AI Developer Intern Co-op</t>
+          <t>Software Engineer 1 Co-op, Anvi</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -2704,24 +2752,24 @@
       <c r="E73" s="4" t="inlineStr"/>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Planview</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>AI and Compiler Engineering Graduate Intern</t>
+          <t>Software Engineer 1 Co-op, Hub</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2732,24 +2780,24 @@
       <c r="E74" s="4" t="inlineStr"/>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Sep 9, 2026</t>
+          <t>Sep 22, 2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Rivian and Volkswagen Group Technologies</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Intern, Vehicle Controls</t>
+          <t>Software Engineering Intern (Spring 2027)</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2760,24 +2808,24 @@
       <c r="E75" s="4" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Sep 8, 2026</t>
+          <t>Sep 21, 2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics Co-op, Customer Operations</t>
+          <t>Investment Risk Analytics Solutions Co-op Intern</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2788,24 +2836,24 @@
       <c r="E76" s="4" t="inlineStr"/>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Sep 5, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Data Analytics Intern</t>
+          <t>AI and Automation Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2816,24 +2864,24 @@
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer in Data Intern</t>
+          <t>Technology Solutions Engineer Co-op/Intern</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2844,24 +2892,24 @@
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Platform</t>
+          <t>Software Engineer Co-op Intern, Investment Tech/Data &amp; Analytics</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2872,24 +2920,24 @@
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>British Columbia Investment</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Data Engineer Intern</t>
+          <t>Software Engineer Co-op Intern</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Victoria, BC</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2900,24 +2948,24 @@
       <c r="E80" s="4" t="inlineStr"/>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 17, 2026</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Full-Stack</t>
+          <t>IT Co-op, Cloud Platforms, Tools &amp; Automation</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2928,24 +2976,24 @@
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>A Thinking Ape</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Data Engineer Intern</t>
+          <t>Software Development Engineer Co-op</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Toronto, ON / Remote, Canada</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2956,24 +3004,24 @@
       <c r="E82" s="4" t="inlineStr"/>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 15, 2026</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Test Developer Co-op</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2984,24 +3032,24 @@
       <c r="E83" s="4" t="inlineStr"/>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Sep 4, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>AltaML</t>
+          <t>Visier Solutions</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Associate Software Developer</t>
+          <t>Software Developer Co-op</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / Edmonton, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -3012,24 +3060,24 @@
       <c r="E84" s="4" t="inlineStr"/>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 11, 2026</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>Mackenzie Investments</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Sensor Fusion Defence Intern</t>
+          <t>Winter Intern, Investment Management, Multi-Asset</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3040,19 +3088,19 @@
       <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 10, 2026</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Defense Engineer Intern</t>
+          <t>Measurement Intern</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -3068,19 +3116,19 @@
       <c r="E86" s="4" t="inlineStr"/>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Hexagon AB</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Geomatics Engineer Intern</t>
+          <t>Specialty Chemicals Engineering &amp; Technical Analyst</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -3096,24 +3144,24 @@
       <c r="E87" s="4" t="inlineStr"/>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Kinaxis</t>
+          <t>SECURE</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Developer Intern Co-op, Machine Learning</t>
+          <t>Software Developer Intern</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -3124,24 +3172,24 @@
       <c r="E88" s="4" t="inlineStr"/>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>North American Construction Group</t>
+          <t>Intact</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Developer Co-op</t>
+          <t>AI Developer Intern Co-op</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Acheson, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3152,24 +3200,24 @@
       <c r="E89" s="4" t="inlineStr"/>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>Varian</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Software Developer Co-op</t>
+          <t>AI and Compiler Engineering Graduate Intern</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -3180,24 +3228,24 @@
       <c r="E90" s="4" t="inlineStr"/>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Sep 3, 2026</t>
+          <t>Sep 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Rivian and Volkswagen Group Technologies</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern/Co-op</t>
+          <t>Software Engineering Intern, Vehicle Controls</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3208,24 +3256,24 @@
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Sep 1, 2026</t>
+          <t>Sep 8, 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Motorola</t>
+          <t>ATCO</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Data Analyst Co-op</t>
+          <t>Data Analytics Co-op, Customer Operations</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Edmonton, AB</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -3236,24 +3284,24 @@
       <c r="E92" s="4" t="inlineStr"/>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 5, 2026</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>CLEAResult</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Energy Efficiency Analyst Co-op</t>
+          <t>Data Analytics Intern</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Remote, Canada</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -3264,24 +3312,24 @@
       <c r="E93" s="4" t="inlineStr"/>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Aug 24, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Software Engineer in Data Intern</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -3292,24 +3340,24 @@
       <c r="E94" s="4" t="inlineStr"/>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Cloud, Data and AI Intern</t>
+          <t>Software Engineer Intern, Platform</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -3320,24 +3368,24 @@
       <c r="E95" s="4" t="inlineStr"/>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Summer Intern, SAP</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -3348,24 +3396,24 @@
       <c r="E96" s="4" t="inlineStr"/>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Aug 18, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Automation Intern - Software or Computer Engineering Student</t>
+          <t>Software Engineer Intern, Full-Stack</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3376,24 +3424,24 @@
       <c r="E97" s="4" t="inlineStr"/>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>Suncor</t>
+          <t>Super</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Data Science Student</t>
+          <t>Data Engineer Intern</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+          <t>Toronto, ON / Remote, Canada</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -3404,24 +3452,24 @@
       <c r="E98" s="4" t="inlineStr"/>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Aug 17, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>ATCO</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Engineering Co-op, Electric Division</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB / Calgary, AB</t>
+          <t>Edmonton, AB / Toronto, ON / Calgary, AB</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -3432,24 +3480,24 @@
       <c r="E99" s="4" t="inlineStr"/>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>Aug 11, 2026</t>
+          <t>Sep 4, 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>AltaML</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern, Gears of War</t>
+          <t>Associate Software Developer</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB / Edmonton, AB</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -3460,24 +3508,24 @@
       <c r="E100" s="4" t="inlineStr"/>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Aug 6, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Sensor Fusion Defence Intern</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -3488,24 +3536,24 @@
       <c r="E101" s="4" t="inlineStr"/>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>Aug 2, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Onware</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Full Stack Developer, Intern</t>
+          <t>Defense Engineer Intern</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Edmonton, AB</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -3516,24 +3564,24 @@
       <c r="E102" s="4" t="inlineStr"/>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Jul 21, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Hexagon AB</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Risk Analytics Solutions Co-op/Intern</t>
+          <t>Geomatics Engineer Intern</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -3544,24 +3592,24 @@
       <c r="E103" s="4" t="inlineStr"/>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>Kinaxis</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+          <t>Developer Intern Co-op, Machine Learning</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC</t>
+          <t>Remote, Canada</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -3572,24 +3620,24 @@
       <c r="E104" s="4" t="inlineStr"/>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>May 14, 2026</t>
+          <t>Sep 3, 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>British Columbia Investment</t>
+          <t>North American Construction Group</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+          <t>Full Stack Developer Co-op</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Victoria, BC / Vancouver, BC</t>
+          <t>Acheson, AB</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -3600,12 +3648,516 @@
       <c r="E105" s="4" t="inlineStr"/>
       <c r="F105" s="4" t="inlineStr">
         <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>Varian</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Software Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr"/>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>Sep 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>Remarcable</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Full Stack Developer Co-op</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr"/>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern/Co-op</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr"/>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>Sep 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Mackenzie Investments</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Investment Management Intern, Canadian Equities</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr"/>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>Aug 26, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>Motorola</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Data Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr"/>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>CLEAResult</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Energy Efficiency Analyst Co-op</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>Remote, Canada</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr"/>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>Aug 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr"/>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Cloud, Data and AI Intern</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="inlineStr"/>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Summer Intern, SAP</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr"/>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>Aug 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Automation Intern - Software or Computer Engineering Student</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr"/>
+      <c r="F115" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Data Science Student</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>Calgary, AB / St. John's, NL / Fort McMurray, AB</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr"/>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>Aug 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>ATCO</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>Engineering Co-op, Electric Division</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB / Calgary, AB</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr"/>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
+          <t>Aug 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Gears of War</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr"/>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>Aug 6, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr"/>
+      <c r="F119" s="4" t="inlineStr">
+        <is>
+          <t>Aug 2, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>Onware</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Full Stack Developer, Intern</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>Edmonton, AB</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr"/>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>Jul 21, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Risk Analytics Solutions Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr"/>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
           <t>May 14, 2026</t>
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Risk Reporting &amp; Data Co-op/Internship</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr"/>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>British Columbia Investment</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics Engineer Co-op/Intern</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Victoria, BC / Vancouver, BC</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr"/>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>May 14, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F105"/>
+  <autoFilter ref="A1:F123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>